<commit_message>
3rd and 4th day
</commit_message>
<xml_diff>
--- a/12628918.xlsx
+++ b/12628918.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/26b1e7fc98125237/Desktop/CAP776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CAD5F233-E97C-4AC4-99AB-63E79547DBAD}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86298FD9-FAA2-40E0-9AFE-0723CF0C0B89}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="65">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -221,6 +221,15 @@
   </si>
   <si>
     <t>in the evening, apart from my college studies, I studied a software develpoment course.</t>
+  </si>
+  <si>
+    <t>Very Satisfied</t>
+  </si>
+  <si>
+    <t>today I learn git in advance</t>
+  </si>
+  <si>
+    <t>more focus on new skills</t>
   </si>
 </sst>
 </file>
@@ -1138,48 +1147,96 @@
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A9" s="13"/>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="15" t="str">
+      <c r="A9" s="13">
+        <v>46248</v>
+      </c>
+      <c r="B9" s="14">
+        <v>420</v>
+      </c>
+      <c r="C9" s="14">
+        <v>0</v>
+      </c>
+      <c r="D9" s="14">
+        <v>120</v>
+      </c>
+      <c r="E9" s="14">
+        <v>90</v>
+      </c>
+      <c r="F9" s="14">
+        <v>250</v>
+      </c>
+      <c r="G9" s="14">
+        <v>5</v>
+      </c>
+      <c r="H9" s="14">
+        <v>90</v>
+      </c>
+      <c r="I9" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J9" s="15" t="str">
+        <v>970</v>
+      </c>
+      <c r="J9" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K9" s="16"/>
-      <c r="L9" s="16"/>
-      <c r="M9" s="16"/>
-      <c r="N9" s="17"/>
+        <v>470</v>
+      </c>
+      <c r="K9" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L9" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="M9" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N9" s="17" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A10" s="13"/>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="15" t="str">
+      <c r="A10" s="13">
+        <v>46249</v>
+      </c>
+      <c r="B10" s="14">
+        <v>420</v>
+      </c>
+      <c r="C10" s="14">
+        <v>0</v>
+      </c>
+      <c r="D10" s="14">
+        <v>240</v>
+      </c>
+      <c r="E10" s="14">
+        <v>60</v>
+      </c>
+      <c r="F10" s="14">
+        <v>0</v>
+      </c>
+      <c r="G10" s="14">
+        <v>0</v>
+      </c>
+      <c r="H10" s="14">
+        <v>0</v>
+      </c>
+      <c r="I10" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J10" s="15" t="str">
+        <v>720</v>
+      </c>
+      <c r="J10" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K10" s="16"/>
-      <c r="L10" s="16"/>
-      <c r="M10" s="16"/>
-      <c r="N10" s="17"/>
+        <v>720</v>
+      </c>
+      <c r="K10" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L10" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="M10" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N10" s="17" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" s="13"/>

</xml_diff>